<commit_message>
fix(crm): explicita data alternativa do cadastro
</commit_message>
<xml_diff>
--- a/outputs/clientes-destinatarios-sem-frete-2026.xlsx
+++ b/outputs/clientes-destinatarios-sem-frete-2026.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes 2026" sheetId="1" r:id="Rfb7c6debff0d4726"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Clientes 2026" sheetId="1" r:id="R6914366781d04f38"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -194,7 +194,7 @@
     <x:tableColumn id="5" name="E-mail"/>
     <x:tableColumn id="6" name="Telefone fixo"/>
     <x:tableColumn id="7" name="Tipo no CT-e"/>
-    <x:tableColumn id="8" name="Data cadastro"/>
+    <x:tableColumn id="8" name="Data cadastro (ou emissão CT-e)"/>
     <x:tableColumn id="9" name="Primeiro CT-e sem frete"/>
     <x:tableColumn id="10" name="Contato — Nome"/>
     <x:tableColumn id="11" name="Contato — Setor"/>
@@ -504,7 +504,7 @@
         <x:v>Tipo no CT-e</x:v>
       </x:c>
       <x:c r="H11" s="22" t="str">
-        <x:v>Data cadastro</x:v>
+        <x:v>Data cadastro (ou emissão CT-e)</x:v>
       </x:c>
       <x:c r="I11" s="22" t="str">
         <x:v>Primeiro CT-e sem frete</x:v>
@@ -15977,7 +15977,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R32cd98b6f7bc43f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bebe90464f64755"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>